<commit_message>
Export: ID lookup, export report, replace guard
The lookup holds each Export ID's tab, No., title and match key values. The
report counts rows per tab and lists unreadable dates and rows with no No.
An existing Collection Workbook is replaced only when the caller says so.
The LibreOffice harness gains --trace to name the line a runtime error hit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHiQNax3FRSR7QTEokLKWr
</commit_message>
<xml_diff>
--- a/tests/fixtures/MainDatabase.xlsx
+++ b/tests/fixtures/MainDatabase.xlsx
@@ -246,8 +246,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_PosterOralPresentation" displayName="tbl_PosterOralPresentation" ref="B1:M5" headerRowCount="1">
-  <autoFilter ref="B1:M5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_PosterOralPresentation" displayName="tbl_PosterOralPresentation" ref="B1:M6" headerRowCount="1">
+  <autoFilter ref="B1:M6"/>
   <tableColumns count="12">
     <tableColumn id="2" name="No."/>
     <tableColumn id="3" name="Title of Presentation/Topic_x000a__x000a__x000a_"/>
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M5"/>
+  <dimension ref="B1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
@@ -966,6 +966,37 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>Singapore</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Return to work after stroke</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lee Hui Min</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Presented</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>44686</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>44686</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>44687</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Test Work Rehab Day</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Check: name the Main Database rows when a key matches several records
The real Main Database has Media rows repeated with the same title and
outlet; the note now says so instead of only "can't find".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHiQNax3FRSR7QTEokLKWr
</commit_message>
<xml_diff>
--- a/tests/fixtures/MainDatabase.xlsx
+++ b/tests/fixtures/MainDatabase.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J6"/>
+  <dimension ref="B1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1777,6 +1777,40 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>Test Blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7">
+        <f>IF(INDEX(B:B,ROW()-1)="No.",1,INDEX(B:B,ROW()-1)+1)</f>
+        <v/>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tan Wei Ling</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Social Media</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>45627</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Therapy tips video</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TestTube</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://example.com/v</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Export: drop Dropped and undated projects, leave out No., new tab order and layout
- Projects: never export one with a Dropped status or no LOA Start, which
  ends the Applied-with-no-LOA rule.
- Leave the Main Database's No. column out of every tab. The ID lookup
  still keeps each row's No., and Check still compares No. in
  Collection Workbooks exported before this change.
- Order the tabs Projects, Publications, Poster & Oral Presentation,
  Education, Media, Talent Development.
- Lay each tab out for reading: the how-to note in 14-point type in one
  cell merged across the table; a bold 12-point header row in white on
  dark blue; centred, wrapped text with a light grey grid and padded row
  heights; columns at least 16 wide; a custom table style with no row
  stripes, so rows added below the table get the same grid.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHiQNax3FRSR7QTEokLKWr
</commit_message>
<xml_diff>
--- a/tests/fixtures/MainDatabase.xlsx
+++ b/tests/fixtures/MainDatabase.xlsx
@@ -163,8 +163,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_PrjGeneralInfo" displayName="tbl_PrjGeneralInfo" ref="A1:AO10" headerRowCount="1">
-  <autoFilter ref="A1:AO10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_PrjGeneralInfo" displayName="tbl_PrjGeneralInfo" ref="A1:AO11" headerRowCount="1">
+  <autoFilter ref="A1:AO11"/>
   <tableColumns count="41">
     <tableColumn id="1" name="Grant Ref No"/>
     <tableColumn id="2" name="Project Name"/>
@@ -2173,7 +2173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO10"/>
+  <dimension ref="A1:AO11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3592,9 +3592,145 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GRT-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Balance clinic evaluation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Invented project for tests</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Test Fund</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Test Group A</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Intramural</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Balance
+(Test Fund)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Goh Mei Xin</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Goh Mei Xin
+</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Admin Person</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>RA Person</t>
+        </is>
+      </c>
+      <c r="Q11" s="1" t="n">
+        <v>45444</v>
+      </c>
+      <c r="R11" s="1" t="n">
+        <v>46173</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>40000</v>
+      </c>
+      <c r="V11" s="2" t="n">
+        <v>40000</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>CC-TEST</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>IOG-TEST</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>IO-TEST-GRT-010</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>1 RA</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>40000</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>60000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="Y2:Y10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>list_PrjStatus</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>